<commit_message>
Update data in October 2025
</commit_message>
<xml_diff>
--- a/Duncan_Index/Duncan index by FINALSEP23.xlsx
+++ b/Duncan_Index/Duncan index by FINALSEP23.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impservihub-my.sharepoint.com/personal/nicholas_cassidy_improvementservice_org_uk/Documents/CPOP/Duncan_Index/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{C04CD266-B673-4A76-A326-10683D993422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5487D782-FDAE-4C67-AC66-26DF1CEA5329}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{C04CD266-B673-4A76-A326-10683D993422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2577A6F-BB57-4230-924C-16AA1505B8E9}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Intro" sheetId="2" r:id="rId1"/>
@@ -15727,7 +15727,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:L417"/>
+  <dimension ref="A1:K417"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -21740,7 +21740,7 @@
         <v>0.17859918839424799</v>
       </c>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>192</v>
       </c>
@@ -21778,7 +21778,7 @@
         <v>0.22085661975811299</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>193</v>
       </c>
@@ -21819,11 +21819,8 @@
         <f>'CPP Raw Data'!K162*-1</f>
         <v>0.25270882457377503</v>
       </c>
-      <c r="L194">
-        <v>0.30371995699999998</v>
-      </c>
-    </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>194</v>
       </c>
@@ -21864,11 +21861,8 @@
         <f>'CPP Raw Data'!K163*-1</f>
         <v>0.200462549183236</v>
       </c>
-      <c r="L195">
-        <v>0.23764270100000001</v>
-      </c>
-    </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>195</v>
       </c>
@@ -21909,11 +21903,8 @@
         <f>'CPP Raw Data'!K164*-1</f>
         <v>0.22438340063656201</v>
       </c>
-      <c r="L196">
-        <v>0.22548860100000001</v>
-      </c>
-    </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>196</v>
       </c>
@@ -21954,11 +21945,8 @@
         <f>'CPP Raw Data'!K165*-1</f>
         <v>0.17565656811901401</v>
       </c>
-      <c r="L197">
-        <v>0.119984196</v>
-      </c>
-    </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>197</v>
       </c>
@@ -21999,11 +21987,8 @@
         <f>'CPP Raw Data'!K166*-1</f>
         <v>0.186597829585259</v>
       </c>
-      <c r="L198">
-        <v>0.23643059599999999</v>
-      </c>
-    </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>198</v>
       </c>
@@ -22044,11 +22029,8 @@
         <f>'CPP Raw Data'!K167*-1</f>
         <v>0.13951808512411601</v>
       </c>
-      <c r="L199">
-        <v>0.17932595900000001</v>
-      </c>
-    </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>199</v>
       </c>
@@ -22089,11 +22071,8 @@
         <f>'CPP Raw Data'!K168*-1</f>
         <v>0.252015637050235</v>
       </c>
-      <c r="L200">
-        <v>0.30069367800000002</v>
-      </c>
-    </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>200</v>
       </c>
@@ -22134,11 +22113,8 @@
         <f>'CPP Raw Data'!K169*-1</f>
         <v>0.18258335675193399</v>
       </c>
-      <c r="L201">
-        <v>0.25533378899999998</v>
-      </c>
-    </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>201</v>
       </c>
@@ -22179,11 +22155,8 @@
         <f>'CPP Raw Data'!K170*-1</f>
         <v>0.253928488516729</v>
       </c>
-      <c r="L202">
-        <v>0.31304944000000001</v>
-      </c>
-    </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>202</v>
       </c>
@@ -22224,11 +22197,8 @@
         <f>'CPP Raw Data'!K171*-1</f>
         <v>0.166822748980782</v>
       </c>
-      <c r="L203">
-        <v>0.23001612099999999</v>
-      </c>
-    </row>
-    <row r="204" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>203</v>
       </c>
@@ -22269,11 +22239,8 @@
         <f>'CPP Raw Data'!K172*-1</f>
         <v>0.35685298295142198</v>
       </c>
-      <c r="L204">
-        <v>0.36561763200000003</v>
-      </c>
-    </row>
-    <row r="205" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>204</v>
       </c>
@@ -22314,11 +22281,8 @@
         <f>'CPP Raw Data'!K173*-1</f>
         <v>0.40317356345868699</v>
       </c>
-      <c r="L205">
-        <v>0.38362973700000003</v>
-      </c>
-    </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>205</v>
       </c>
@@ -22359,11 +22323,8 @@
         <f>'CPP Raw Data'!K174*-1</f>
         <v>-2.3262108133078399E-2</v>
       </c>
-      <c r="L206">
-        <v>-6.4445503000000001E-2</v>
-      </c>
-    </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>206</v>
       </c>
@@ -22404,11 +22365,8 @@
         <f>'CPP Raw Data'!K175*-1</f>
         <v>0.211217391267956</v>
       </c>
-      <c r="L207">
-        <v>0.25652097699999998</v>
-      </c>
-    </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>207</v>
       </c>
@@ -22449,11 +22407,8 @@
         <f>'CPP Raw Data'!K176*-1</f>
         <v>0.26382578027508802</v>
       </c>
-      <c r="L208">
-        <v>0.32663207700000002</v>
-      </c>
-    </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>208</v>
       </c>
@@ -22494,11 +22449,8 @@
         <f>'CPP Raw Data'!K177*-1</f>
         <v>0.198366875620586</v>
       </c>
-      <c r="L209">
-        <v>0.22242015600000001</v>
-      </c>
-    </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A210">
         <v>209</v>
       </c>
@@ -22539,11 +22491,8 @@
         <f>'CPP Raw Data'!K178*-1</f>
         <v>0.16898214605353701</v>
       </c>
-      <c r="L210">
-        <v>0.18774796299999999</v>
-      </c>
-    </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A211">
         <v>210</v>
       </c>
@@ -22584,11 +22533,8 @@
         <f>'CPP Raw Data'!K179*-1</f>
         <v>0.28863142321747798</v>
       </c>
-      <c r="L211">
-        <v>0.30315756700000002</v>
-      </c>
-    </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A212">
         <v>211</v>
       </c>
@@ -22629,11 +22575,8 @@
         <f>'CPP Raw Data'!K180*-1</f>
         <v>0.18538700301195599</v>
       </c>
-      <c r="L212">
-        <v>0.23930818600000001</v>
-      </c>
-    </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A213">
         <v>212</v>
       </c>
@@ -22674,11 +22617,8 @@
         <f>'CPP Raw Data'!K181*-1</f>
         <v>6.7786779482672102E-2</v>
       </c>
-      <c r="L213">
-        <v>0.112627779</v>
-      </c>
-    </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="214" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A214">
         <v>213</v>
       </c>
@@ -22719,11 +22659,8 @@
         <f>'CPP Raw Data'!K182*-1</f>
         <v>0.27187686255813898</v>
       </c>
-      <c r="L214">
-        <v>0.280187723</v>
-      </c>
-    </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="215" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A215">
         <v>214</v>
       </c>
@@ -22764,11 +22701,8 @@
         <f>'CPP Raw Data'!K183*-1</f>
         <v>0.145385806308621</v>
       </c>
-      <c r="L215">
-        <v>0.20169378499999999</v>
-      </c>
-    </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="216" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A216">
         <v>215</v>
       </c>
@@ -22809,11 +22743,8 @@
         <f>'CPP Raw Data'!K184*-1</f>
         <v>5.0559037489196899E-2</v>
       </c>
-      <c r="L216">
-        <v>9.9942157000000004E-2</v>
-      </c>
-    </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="217" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A217">
         <v>216</v>
       </c>
@@ -22854,11 +22785,8 @@
         <f>'CPP Raw Data'!K185*-1</f>
         <v>0.21395126401644801</v>
       </c>
-      <c r="L217">
-        <v>0.23305498499999999</v>
-      </c>
-    </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="218" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A218">
         <v>217</v>
       </c>
@@ -22899,11 +22827,8 @@
         <f>'CPP Raw Data'!K186*-1</f>
         <v>0.252791136410494</v>
       </c>
-      <c r="L218">
-        <v>0.33996794600000002</v>
-      </c>
-    </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="219" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A219">
         <v>218</v>
       </c>
@@ -22944,11 +22869,8 @@
         <f>'CPP Raw Data'!K187*-1</f>
         <v>0.16033683423954601</v>
       </c>
-      <c r="L219">
-        <v>0.21718216300000001</v>
-      </c>
-    </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="220" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A220">
         <v>219</v>
       </c>
@@ -22989,11 +22911,8 @@
         <f>'CPP Raw Data'!K188*-1</f>
         <v>9.5802041409070102E-2</v>
       </c>
-      <c r="L220">
-        <v>-4.2589864999999998E-2</v>
-      </c>
-    </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="221" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A221">
         <v>220</v>
       </c>
@@ -23034,11 +22953,8 @@
         <f>'CPP Raw Data'!K189*-1</f>
         <v>0.23957479755090499</v>
       </c>
-      <c r="L221">
-        <v>0.29941983900000002</v>
-      </c>
-    </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="222" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A222">
         <v>221</v>
       </c>
@@ -23079,11 +22995,8 @@
         <f>'CPP Raw Data'!K190*-1</f>
         <v>0.175223027866419</v>
       </c>
-      <c r="L222">
-        <v>0.24323082700000001</v>
-      </c>
-    </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="223" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A223">
         <v>222</v>
       </c>
@@ -23124,11 +23037,8 @@
         <f>'CPP Raw Data'!K191*-1</f>
         <v>0.30667239096600402</v>
       </c>
-      <c r="L223">
-        <v>0.32520884</v>
-      </c>
-    </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="224" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A224">
         <v>223</v>
       </c>
@@ -23169,11 +23079,8 @@
         <f>'CPP Raw Data'!K192*-1</f>
         <v>0.175786508161456</v>
       </c>
-      <c r="L224">
-        <v>0.19679476400000001</v>
-      </c>
-    </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A225">
         <v>224</v>
       </c>
@@ -23214,11 +23121,8 @@
         <f>'CPP Raw Data'!K193*-1</f>
         <v>0.180205532824464</v>
       </c>
-      <c r="L225">
-        <v>0.248281851</v>
-      </c>
-    </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A226">
         <v>225</v>
       </c>
@@ -23259,11 +23163,8 @@
         <f>'CPP Raw Data'!K194*-1</f>
         <v>0.29281022322054001</v>
       </c>
-      <c r="L226">
-        <v>0.30057064900000002</v>
-      </c>
-    </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A227">
         <v>226</v>
       </c>
@@ -23304,11 +23205,8 @@
         <f>'CPP Raw Data'!K195*-1</f>
         <v>0.279302045417676</v>
       </c>
-      <c r="L227">
-        <v>0.26550564500000001</v>
-      </c>
-    </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A228">
         <v>227</v>
       </c>
@@ -23349,11 +23247,8 @@
         <f>'CPP Raw Data'!K196*-1</f>
         <v>0.26716569053443401</v>
       </c>
-      <c r="L228">
-        <v>0.242814841</v>
-      </c>
-    </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A229">
         <v>228</v>
       </c>
@@ -23394,11 +23289,8 @@
         <f>'CPP Raw Data'!K197*-1</f>
         <v>0.19670163588779299</v>
       </c>
-      <c r="L229">
-        <v>5.2768502000000002E-2</v>
-      </c>
-    </row>
-    <row r="230" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A230">
         <v>229</v>
       </c>
@@ -23439,11 +23331,8 @@
         <f>'CPP Raw Data'!K198*-1</f>
         <v>0.20324796660323499</v>
       </c>
-      <c r="L230">
-        <v>0.24638966200000001</v>
-      </c>
-    </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A231">
         <v>230</v>
       </c>
@@ -23484,11 +23373,8 @@
         <f>'CPP Raw Data'!K199*-1</f>
         <v>0.16053750494303801</v>
       </c>
-      <c r="L231">
-        <v>0.16670807900000001</v>
-      </c>
-    </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="232" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A232">
         <v>231</v>
       </c>
@@ -23529,11 +23415,8 @@
         <f>'CPP Raw Data'!K200*-1</f>
         <v>0.25227948900353803</v>
       </c>
-      <c r="L232">
-        <v>0.29071930800000001</v>
-      </c>
-    </row>
-    <row r="233" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="233" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A233">
         <v>232</v>
       </c>
@@ -23574,11 +23457,8 @@
         <f>'CPP Raw Data'!K201*-1</f>
         <v>0.21931233269196501</v>
       </c>
-      <c r="L233">
-        <v>0.264699248</v>
-      </c>
-    </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="234" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A234">
         <v>233</v>
       </c>
@@ -23619,11 +23499,8 @@
         <f>'CPP Raw Data'!K202*-1</f>
         <v>0.28029157069573102</v>
       </c>
-      <c r="L234">
-        <v>0.31365848000000002</v>
-      </c>
-    </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A235">
         <v>234</v>
       </c>
@@ -23664,11 +23541,8 @@
         <f>'CPP Raw Data'!K203*-1</f>
         <v>0.178639988081115</v>
       </c>
-      <c r="L235">
-        <v>0.229746802</v>
-      </c>
-    </row>
-    <row r="236" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A236">
         <v>235</v>
       </c>
@@ -23709,11 +23583,8 @@
         <f>'CPP Raw Data'!K204*-1</f>
         <v>0.39022993812909801</v>
       </c>
-      <c r="L236">
-        <v>0.36162846700000001</v>
-      </c>
-    </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A237">
         <v>236</v>
       </c>
@@ -23754,11 +23625,8 @@
         <f>'CPP Raw Data'!K205*-1</f>
         <v>0.43072067589704599</v>
       </c>
-      <c r="L237">
-        <v>0.3607996</v>
-      </c>
-    </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A238">
         <v>237</v>
       </c>
@@ -23799,11 +23667,8 @@
         <f>'CPP Raw Data'!K206*-1</f>
         <v>-7.18239871015669E-3</v>
       </c>
-      <c r="L238">
-        <v>2.1398357E-2</v>
-      </c>
-    </row>
-    <row r="239" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A239">
         <v>238</v>
       </c>
@@ -23844,11 +23709,8 @@
         <f>'CPP Raw Data'!K207*-1</f>
         <v>0.23313164931661301</v>
       </c>
-      <c r="L239">
-        <v>0.25696376399999998</v>
-      </c>
-    </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A240">
         <v>239</v>
       </c>
@@ -23889,11 +23751,8 @@
         <f>'CPP Raw Data'!K208*-1</f>
         <v>0.31402528468243002</v>
       </c>
-      <c r="L240">
-        <v>0.30301345000000002</v>
-      </c>
-    </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="241" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A241">
         <v>240</v>
       </c>
@@ -23934,11 +23793,8 @@
         <f>'CPP Raw Data'!K209*-1</f>
         <v>0.237015694075701</v>
       </c>
-      <c r="L241">
-        <v>0.23688393299999999</v>
-      </c>
-    </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="242" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A242">
         <v>241</v>
       </c>
@@ -23979,11 +23835,8 @@
         <f>'CPP Raw Data'!K210*-1</f>
         <v>0.20770641197895801</v>
       </c>
-      <c r="L242">
-        <v>0.15361174699999999</v>
-      </c>
-    </row>
-    <row r="243" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="243" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A243">
         <v>242</v>
       </c>
@@ -24024,11 +23877,8 @@
         <f>'CPP Raw Data'!K211*-1</f>
         <v>0.323173037582625</v>
       </c>
-      <c r="L243">
-        <v>0.31520254399999997</v>
-      </c>
-    </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="244" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A244">
         <v>243</v>
       </c>
@@ -24069,11 +23919,8 @@
         <f>'CPP Raw Data'!K212*-1</f>
         <v>0.218891112739421</v>
       </c>
-      <c r="L244">
-        <v>0.20941750100000001</v>
-      </c>
-    </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="245" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A245">
         <v>244</v>
       </c>
@@ -24114,11 +23961,8 @@
         <f>'CPP Raw Data'!K213*-1</f>
         <v>9.0953645745549302E-2</v>
       </c>
-      <c r="L245">
-        <v>0.114773425</v>
-      </c>
-    </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="246" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A246">
         <v>245</v>
       </c>
@@ -24159,11 +24003,8 @@
         <f>'CPP Raw Data'!K214*-1</f>
         <v>0.27393673565847498</v>
       </c>
-      <c r="L246">
-        <v>0.28203809000000002</v>
-      </c>
-    </row>
-    <row r="247" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="247" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A247">
         <v>246</v>
       </c>
@@ -24204,11 +24045,8 @@
         <f>'CPP Raw Data'!K215*-1</f>
         <v>0.184089032839484</v>
       </c>
-      <c r="L247">
-        <v>0.192016933</v>
-      </c>
-    </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="248" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A248">
         <v>247</v>
       </c>
@@ -24249,11 +24087,8 @@
         <f>'CPP Raw Data'!K216*-1</f>
         <v>8.5962136523555693E-2</v>
       </c>
-      <c r="L248">
-        <v>1.1214435E-2</v>
-      </c>
-    </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="249" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A249">
         <v>248</v>
       </c>
@@ -24294,11 +24129,8 @@
         <f>'CPP Raw Data'!K217*-1</f>
         <v>0.245484606109518</v>
       </c>
-      <c r="L249">
-        <v>0.239028247</v>
-      </c>
-    </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A250">
         <v>249</v>
       </c>
@@ -24339,11 +24171,8 @@
         <f>'CPP Raw Data'!K218*-1</f>
         <v>0.28138133023133899</v>
       </c>
-      <c r="L250">
-        <v>0.331775231</v>
-      </c>
-    </row>
-    <row r="251" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A251">
         <v>250</v>
       </c>
@@ -24384,11 +24213,8 @@
         <f>'CPP Raw Data'!K219*-1</f>
         <v>0.17749720676387201</v>
       </c>
-      <c r="L251">
-        <v>0.22137279200000001</v>
-      </c>
-    </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="252" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A252">
         <v>251</v>
       </c>
@@ -24429,11 +24255,8 @@
         <f>'CPP Raw Data'!K220*-1</f>
         <v>7.8391283902466094E-2</v>
       </c>
-      <c r="L252">
-        <v>8.6313850000000001E-3</v>
-      </c>
-    </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="253" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A253">
         <v>252</v>
       </c>
@@ -24474,11 +24297,8 @@
         <f>'CPP Raw Data'!K221*-1</f>
         <v>0.26455697876990902</v>
       </c>
-      <c r="L253">
-        <v>0.29739148599999998</v>
-      </c>
-    </row>
-    <row r="254" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="254" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A254">
         <v>253</v>
       </c>
@@ -24519,11 +24339,8 @@
         <f>'CPP Raw Data'!K222*-1</f>
         <v>0.222987442600559</v>
       </c>
-      <c r="L254">
-        <v>0.21606766899999999</v>
-      </c>
-    </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="255" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A255">
         <v>254</v>
       </c>
@@ -24564,11 +24381,8 @@
         <f>'CPP Raw Data'!K223*-1</f>
         <v>0.31750168481667101</v>
       </c>
-      <c r="L255">
-        <v>0.31827307500000002</v>
-      </c>
-    </row>
-    <row r="256" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="256" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A256">
         <v>255</v>
       </c>
@@ -24609,11 +24423,8 @@
         <f>'CPP Raw Data'!K224*-1</f>
         <v>0.20226575060045299</v>
       </c>
-      <c r="L256">
-        <v>0.17992073</v>
-      </c>
-    </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="257" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A257">
         <v>256</v>
       </c>
@@ -24654,11 +24465,8 @@
         <f>'CPP Raw Data'!K225*-1</f>
         <v>0.200173542613031</v>
       </c>
-      <c r="L257">
-        <v>0.22422614699999999</v>
-      </c>
-    </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="258" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A258">
         <v>257</v>
       </c>
@@ -24699,11 +24507,8 @@
         <f>'CPP Raw Data'!K226*-1</f>
         <v>0.29679354251559398</v>
       </c>
-      <c r="L258">
-        <v>0.30166744699999998</v>
-      </c>
-    </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="259" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A259">
         <v>258</v>
       </c>
@@ -24744,11 +24549,8 @@
         <f>'CPP Raw Data'!K227*-1</f>
         <v>0.29233448577280702</v>
       </c>
-      <c r="L259">
-        <v>0.24815983599999999</v>
-      </c>
-    </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="260" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A260">
         <v>259</v>
       </c>
@@ -24789,11 +24591,8 @@
         <f>'CPP Raw Data'!K228*-1</f>
         <v>0.26964312542098001</v>
       </c>
-      <c r="L260">
-        <v>0.27168714599999999</v>
-      </c>
-    </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="261" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A261">
         <v>260</v>
       </c>
@@ -24834,11 +24633,8 @@
         <f>'CPP Raw Data'!K229*-1</f>
         <v>0.196071976823704</v>
       </c>
-      <c r="L261">
-        <v>8.9093108000000004E-2</v>
-      </c>
-    </row>
-    <row r="262" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="262" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A262">
         <v>261</v>
       </c>
@@ -24879,11 +24675,8 @@
         <f>'CPP Raw Data'!K230*-1</f>
         <v>0.198884670547541</v>
       </c>
-      <c r="L262">
-        <v>0.19628853900000001</v>
-      </c>
-    </row>
-    <row r="263" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="263" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A263">
         <v>262</v>
       </c>
@@ -24924,11 +24717,8 @@
         <f>'CPP Raw Data'!K231*-1</f>
         <v>0.18386662466996401</v>
       </c>
-      <c r="L263">
-        <v>0.15705888000000001</v>
-      </c>
-    </row>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="264" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A264">
         <v>263</v>
       </c>
@@ -24969,11 +24759,8 @@
         <f>'CPP Raw Data'!K232*-1</f>
         <v>0.26631289391803697</v>
       </c>
-      <c r="L264">
-        <v>0.31129586799999998</v>
-      </c>
-    </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="265" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A265">
         <v>264</v>
       </c>
@@ -25014,11 +24801,8 @@
         <f>'CPP Raw Data'!K233*-1</f>
         <v>0.223100922965937</v>
       </c>
-      <c r="L265">
-        <v>0.245160712</v>
-      </c>
-    </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="266" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A266">
         <v>265</v>
       </c>
@@ -25059,11 +24843,8 @@
         <f>'CPP Raw Data'!K234*-1</f>
         <v>0.29363993500783903</v>
       </c>
-      <c r="L266">
-        <v>0.33421303499999999</v>
-      </c>
-    </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="267" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A267">
         <v>266</v>
       </c>
@@ -25104,11 +24885,8 @@
         <f>'CPP Raw Data'!K235*-1</f>
         <v>0.193882067646615</v>
       </c>
-      <c r="L267">
-        <v>0.21319803200000001</v>
-      </c>
-    </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="268" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A268">
         <v>267</v>
       </c>
@@ -25149,11 +24927,8 @@
         <f>'CPP Raw Data'!K236*-1</f>
         <v>0.39411050574075801</v>
       </c>
-      <c r="L268">
-        <v>0.41185737700000002</v>
-      </c>
-    </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="269" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A269">
         <v>268</v>
       </c>
@@ -25194,11 +24969,8 @@
         <f>'CPP Raw Data'!K237*-1</f>
         <v>0.43301133433660899</v>
       </c>
-      <c r="L269">
-        <v>0.36901840400000002</v>
-      </c>
-    </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="270" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A270">
         <v>269</v>
       </c>
@@ -25239,11 +25011,8 @@
         <f>'CPP Raw Data'!K238*-1</f>
         <v>2.4725283285477899E-2</v>
       </c>
-      <c r="L270">
-        <v>3.1573331000000003E-2</v>
-      </c>
-    </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="271" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A271">
         <v>270</v>
       </c>
@@ -25284,11 +25053,8 @@
         <f>'CPP Raw Data'!K239*-1</f>
         <v>0.22874069698250199</v>
       </c>
-      <c r="L271">
-        <v>0.242747873</v>
-      </c>
-    </row>
-    <row r="272" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="272" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A272">
         <v>271</v>
       </c>
@@ -25329,11 +25095,8 @@
         <f>'CPP Raw Data'!K240*-1</f>
         <v>0.32533578116932899</v>
       </c>
-      <c r="L272">
-        <v>0.30139855900000001</v>
-      </c>
-    </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="273" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A273">
         <v>272</v>
       </c>
@@ -25374,11 +25137,8 @@
         <f>'CPP Raw Data'!K241*-1</f>
         <v>0.24938274806531499</v>
       </c>
-      <c r="L273">
-        <v>0.21521275500000001</v>
-      </c>
-    </row>
-    <row r="274" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="274" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A274">
         <v>273</v>
       </c>
@@ -25419,11 +25179,8 @@
         <f>'CPP Raw Data'!K242*-1</f>
         <v>0.22178937492713399</v>
       </c>
-      <c r="L274">
-        <v>0.192535066</v>
-      </c>
-    </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="275" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A275">
         <v>274</v>
       </c>
@@ -25464,11 +25221,8 @@
         <f>'CPP Raw Data'!K243*-1</f>
         <v>0.34121173502576502</v>
       </c>
-      <c r="L275">
-        <v>0.28450252399999998</v>
-      </c>
-    </row>
-    <row r="276" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="276" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A276">
         <v>275</v>
       </c>
@@ -25509,11 +25263,8 @@
         <f>'CPP Raw Data'!K244*-1</f>
         <v>0.22514922773693799</v>
       </c>
-      <c r="L276">
-        <v>0.19442004199999999</v>
-      </c>
-    </row>
-    <row r="277" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="277" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A277">
         <v>276</v>
       </c>
@@ -25554,11 +25305,8 @@
         <f>'CPP Raw Data'!K245*-1</f>
         <v>0.11813634788531099</v>
       </c>
-      <c r="L277">
-        <v>9.7188013000000004E-2</v>
-      </c>
-    </row>
-    <row r="278" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="278" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A278">
         <v>277</v>
       </c>
@@ -25599,11 +25347,8 @@
         <f>'CPP Raw Data'!K246*-1</f>
         <v>0.29453064788003802</v>
       </c>
-      <c r="L278">
-        <v>0.27591796400000002</v>
-      </c>
-    </row>
-    <row r="279" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="279" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A279">
         <v>278</v>
       </c>
@@ -25644,11 +25389,8 @@
         <f>'CPP Raw Data'!K247*-1</f>
         <v>0.188690065310961</v>
       </c>
-      <c r="L279">
-        <v>0.20282229700000001</v>
-      </c>
-    </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="280" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A280">
         <v>279</v>
       </c>
@@ -25689,11 +25431,8 @@
         <f>'CPP Raw Data'!K248*-1</f>
         <v>0.12371605114699701</v>
       </c>
-      <c r="L280">
-        <v>5.7498116000000002E-2</v>
-      </c>
-    </row>
-    <row r="281" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="281" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A281">
         <v>280</v>
       </c>
@@ -25734,11 +25473,8 @@
         <f>'CPP Raw Data'!K249*-1</f>
         <v>0.23740107747151201</v>
       </c>
-      <c r="L281">
-        <v>0.239423738</v>
-      </c>
-    </row>
-    <row r="282" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="282" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A282">
         <v>281</v>
       </c>
@@ -25779,11 +25515,8 @@
         <f>'CPP Raw Data'!K250*-1</f>
         <v>0.31431457487164799</v>
       </c>
-      <c r="L282">
-        <v>0.34594270500000002</v>
-      </c>
-    </row>
-    <row r="283" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="283" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A283">
         <v>282</v>
       </c>
@@ -25824,11 +25557,8 @@
         <f>'CPP Raw Data'!K251*-1</f>
         <v>0.19385832002051201</v>
       </c>
-      <c r="L283">
-        <v>0.21284253</v>
-      </c>
-    </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="284" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A284">
         <v>283</v>
       </c>
@@ -25869,11 +25599,8 @@
         <f>'CPP Raw Data'!K252*-1</f>
         <v>8.2072320650595304E-2</v>
       </c>
-      <c r="L284">
-        <v>9.4800512000000003E-2</v>
-      </c>
-    </row>
-    <row r="285" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="285" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A285">
         <v>284</v>
       </c>
@@ -25914,11 +25641,8 @@
         <f>'CPP Raw Data'!K253*-1</f>
         <v>0.29714634224472602</v>
       </c>
-      <c r="L285">
-        <v>0.29639921299999999</v>
-      </c>
-    </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="286" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A286">
         <v>285</v>
       </c>
@@ -25959,11 +25683,8 @@
         <f>'CPP Raw Data'!K254*-1</f>
         <v>0.235244903305905</v>
       </c>
-      <c r="L286">
-        <v>0.24257035699999999</v>
-      </c>
-    </row>
-    <row r="287" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="287" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A287">
         <v>286</v>
       </c>
@@ -26004,11 +25725,8 @@
         <f>'CPP Raw Data'!K255*-1</f>
         <v>0.32177021226651398</v>
       </c>
-      <c r="L287">
-        <v>0.33271719</v>
-      </c>
-    </row>
-    <row r="288" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="288" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A288">
         <v>287</v>
       </c>
@@ -26049,11 +25767,8 @@
         <f>'CPP Raw Data'!K256*-1</f>
         <v>0.208402699009127</v>
       </c>
-      <c r="L288">
-        <v>0.181149433</v>
-      </c>
-    </row>
-    <row r="289" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="289" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A289">
         <v>288</v>
       </c>
@@ -26094,11 +25809,8 @@
         <f>'CPP Raw Data'!K257*-1</f>
         <v>0.219574864790927</v>
       </c>
-      <c r="L289">
-        <v>0.21721896900000001</v>
-      </c>
-    </row>
-    <row r="290" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="290" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A290">
         <v>289</v>
       </c>
@@ -26139,11 +25851,8 @@
         <f>'CPP Raw Data'!K258*-1</f>
         <v>0.31192463073061599</v>
       </c>
-      <c r="L290">
-        <v>-7.3980269999999997E-3</v>
-      </c>
-    </row>
-    <row r="291" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="291" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A291">
         <v>290</v>
       </c>
@@ -26184,11 +25893,8 @@
         <f>'CPP Raw Data'!K259*-1</f>
         <v>0.293603692096642</v>
       </c>
-      <c r="L291">
-        <v>5.8058084000000003E-2</v>
-      </c>
-    </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="292" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A292">
         <v>291</v>
       </c>
@@ -26229,11 +25935,8 @@
         <f>'CPP Raw Data'!K260*-1</f>
         <v>0.26695675542938502</v>
       </c>
-      <c r="L292">
-        <v>-8.4992600000000001E-2</v>
-      </c>
-    </row>
-    <row r="293" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="293" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A293">
         <v>292</v>
       </c>
@@ -26274,11 +25977,8 @@
         <f>'CPP Raw Data'!K261*-1</f>
         <v>0.200002687023033</v>
       </c>
-      <c r="L293">
-        <v>-5.5224233999999997E-2</v>
-      </c>
-    </row>
-    <row r="294" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="294" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A294">
         <v>293</v>
       </c>
@@ -26319,11 +26019,8 @@
         <f>'CPP Raw Data'!K262*-1</f>
         <v>0.20580234414791099</v>
       </c>
-      <c r="L294">
-        <v>0.14843672499999999</v>
-      </c>
-    </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="295" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A295">
         <v>294</v>
       </c>
@@ -26364,11 +26061,8 @@
         <f>'CPP Raw Data'!K263*-1</f>
         <v>0.203639048658493</v>
       </c>
-      <c r="L295">
-        <v>5.3387080000000003E-2</v>
-      </c>
-    </row>
-    <row r="296" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="296" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A296">
         <v>295</v>
       </c>
@@ -26409,11 +26103,8 @@
         <f>'CPP Raw Data'!K264*-1</f>
         <v>0.28227775709385</v>
       </c>
-      <c r="L296">
-        <v>3.8199877E-2</v>
-      </c>
-    </row>
-    <row r="297" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="297" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A297">
         <v>296</v>
       </c>
@@ -26454,11 +26145,8 @@
         <f>'CPP Raw Data'!K265*-1</f>
         <v>0.245755053713372</v>
       </c>
-      <c r="L297">
-        <v>-4.7923618000000001E-2</v>
-      </c>
-    </row>
-    <row r="298" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="298" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A298">
         <v>297</v>
       </c>
@@ -26499,11 +26187,8 @@
         <f>'CPP Raw Data'!K266*-1</f>
         <v>0.31164094618764898</v>
       </c>
-      <c r="L298">
-        <v>-0.16044254399999999</v>
-      </c>
-    </row>
-    <row r="299" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="299" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A299">
         <v>298</v>
       </c>
@@ -26544,11 +26229,8 @@
         <f>'CPP Raw Data'!K267*-1</f>
         <v>0.21169935757525199</v>
       </c>
-      <c r="L299">
-        <v>6.0769266000000002E-2</v>
-      </c>
-    </row>
-    <row r="300" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="300" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A300">
         <v>299</v>
       </c>
@@ -26589,11 +26271,8 @@
         <f>'CPP Raw Data'!K268*-1</f>
         <v>0.39699897541434198</v>
       </c>
-      <c r="L300">
-        <v>-4.8885200000000001E-4</v>
-      </c>
-    </row>
-    <row r="301" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="301" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A301">
         <v>300</v>
       </c>
@@ -26634,11 +26313,8 @@
         <f>'CPP Raw Data'!K269*-1</f>
         <v>0.43270554671918798</v>
       </c>
-      <c r="L301">
-        <v>6.9452849999999998E-3</v>
-      </c>
-    </row>
-    <row r="302" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="302" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A302">
         <v>301</v>
       </c>
@@ -26679,11 +26355,8 @@
         <f>'CPP Raw Data'!K270*-1</f>
         <v>6.0739015045153402E-2</v>
       </c>
-      <c r="L302">
-        <v>3.5772891000000001E-2</v>
-      </c>
-    </row>
-    <row r="303" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="303" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A303">
         <v>302</v>
       </c>
@@ -26724,11 +26397,8 @@
         <f>'CPP Raw Data'!K271*-1</f>
         <v>0.23967857082479499</v>
       </c>
-      <c r="L303">
-        <v>4.0285968999999998E-2</v>
-      </c>
-    </row>
-    <row r="304" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="304" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A304">
         <v>303</v>
       </c>
@@ -26769,11 +26439,8 @@
         <f>'CPP Raw Data'!K272*-1</f>
         <v>0.338235799699941</v>
       </c>
-      <c r="L304">
-        <v>0.106626417</v>
-      </c>
-    </row>
-    <row r="305" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="305" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A305">
         <v>304</v>
       </c>
@@ -26814,11 +26481,8 @@
         <f>'CPP Raw Data'!K273*-1</f>
         <v>0.256717597621062</v>
       </c>
-      <c r="L305">
-        <v>8.4851699000000003E-2</v>
-      </c>
-    </row>
-    <row r="306" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="306" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A306">
         <v>305</v>
       </c>
@@ -26859,11 +26523,8 @@
         <f>'CPP Raw Data'!K274*-1</f>
         <v>0.232182200132065</v>
       </c>
-      <c r="L306">
-        <v>-6.1470481E-2</v>
-      </c>
-    </row>
-    <row r="307" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="307" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A307">
         <v>306</v>
       </c>
@@ -26904,11 +26565,8 @@
         <f>'CPP Raw Data'!K275*-1</f>
         <v>0.35041356521263201</v>
       </c>
-      <c r="L307">
-        <v>0.19884341999999999</v>
-      </c>
-    </row>
-    <row r="308" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="308" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A308">
         <v>307</v>
       </c>
@@ -26949,11 +26607,8 @@
         <f>'CPP Raw Data'!K276*-1</f>
         <v>0.227318332990711</v>
       </c>
-      <c r="L308">
-        <v>-0.108023929</v>
-      </c>
-    </row>
-    <row r="309" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="309" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A309">
         <v>308</v>
       </c>
@@ -26994,11 +26649,8 @@
         <f>'CPP Raw Data'!K277*-1</f>
         <v>0.146229782921727</v>
       </c>
-      <c r="L309">
-        <v>8.6213053999999997E-2</v>
-      </c>
-    </row>
-    <row r="310" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="310" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A310">
         <v>309</v>
       </c>
@@ -27039,11 +26691,8 @@
         <f>'CPP Raw Data'!K278*-1</f>
         <v>0.29868269233237799</v>
       </c>
-      <c r="L310">
-        <v>-7.7124180000000004E-3</v>
-      </c>
-    </row>
-    <row r="311" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="311" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A311">
         <v>310</v>
       </c>
@@ -27084,11 +26733,8 @@
         <f>'CPP Raw Data'!K279*-1</f>
         <v>0.19755332738805401</v>
       </c>
-      <c r="L311">
-        <v>1.3526144E-2</v>
-      </c>
-    </row>
-    <row r="312" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="312" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A312">
         <v>311</v>
       </c>
@@ -27129,11 +26775,8 @@
         <f>'CPP Raw Data'!K280*-1</f>
         <v>0.17408658786381601</v>
       </c>
-      <c r="L312">
-        <v>0.152271084</v>
-      </c>
-    </row>
-    <row r="313" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="313" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A313">
         <v>312</v>
       </c>
@@ -27174,11 +26817,8 @@
         <f>'CPP Raw Data'!K281*-1</f>
         <v>0.25359851822833301</v>
       </c>
-      <c r="L313">
-        <v>9.4285153999999996E-2</v>
-      </c>
-    </row>
-    <row r="314" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="314" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A314">
         <v>313</v>
       </c>
@@ -27219,11 +26859,8 @@
         <f>'CPP Raw Data'!K282*-1</f>
         <v>0.323548865020586</v>
       </c>
-      <c r="L314">
-        <v>0.100081012</v>
-      </c>
-    </row>
-    <row r="315" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="315" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A315">
         <v>314</v>
       </c>
@@ -27264,11 +26901,8 @@
         <f>'CPP Raw Data'!K283*-1</f>
         <v>0.20559735624577499</v>
       </c>
-      <c r="L315">
-        <v>4.4013680000000001E-3</v>
-      </c>
-    </row>
-    <row r="316" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="316" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A316">
         <v>315</v>
       </c>
@@ -27309,11 +26943,8 @@
         <f>'CPP Raw Data'!K284*-1</f>
         <v>8.1784642407645394E-2</v>
       </c>
-      <c r="L316">
-        <v>6.2753054000000003E-2</v>
-      </c>
-    </row>
-    <row r="317" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="317" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A317">
         <v>316</v>
       </c>
@@ -27354,11 +26985,8 @@
         <f>'CPP Raw Data'!K285*-1</f>
         <v>0.29621408822041301</v>
       </c>
-      <c r="L317">
-        <v>-1.3674921E-2</v>
-      </c>
-    </row>
-    <row r="318" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="318" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A318">
         <v>317</v>
       </c>
@@ -27399,11 +27027,8 @@
         <f>'CPP Raw Data'!K286*-1</f>
         <v>0.241427583524327</v>
       </c>
-      <c r="L318">
-        <v>4.5761746999999998E-2</v>
-      </c>
-    </row>
-    <row r="319" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="319" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A319">
         <v>318</v>
       </c>
@@ -27444,11 +27069,8 @@
         <f>'CPP Raw Data'!K287*-1</f>
         <v>0.34280394704346001</v>
       </c>
-      <c r="L319">
-        <v>0.22177375099999999</v>
-      </c>
-    </row>
-    <row r="320" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="320" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A320">
         <v>319</v>
       </c>
@@ -27489,11 +27111,8 @@
         <f>'CPP Raw Data'!K288*-1</f>
         <v>0.20844600956965501</v>
       </c>
-      <c r="L320">
-        <v>7.9089193000000002E-2</v>
-      </c>
-    </row>
-    <row r="321" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="321" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A321">
         <v>320</v>
       </c>
@@ -27534,11 +27153,8 @@
         <f>'CPP Raw Data'!K289*-1</f>
         <v>0.23594730528841301</v>
       </c>
-      <c r="L321">
-        <v>8.6913569999999996E-2</v>
-      </c>
-    </row>
-    <row r="322" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="322" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A322">
         <v>321</v>
       </c>
@@ -27579,11 +27195,8 @@
         <f>'CPP Raw Data'!K290*-1</f>
         <v>0.32637234988046299</v>
       </c>
-      <c r="L322">
-        <v>0.331896839</v>
-      </c>
-    </row>
-    <row r="323" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="323" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A323">
         <v>322</v>
       </c>
@@ -27624,11 +27237,8 @@
         <f>'CPP Raw Data'!K291*-1</f>
         <v>0.29194231605017701</v>
       </c>
-      <c r="L323">
-        <v>0.20305654100000001</v>
-      </c>
-    </row>
-    <row r="324" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="324" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A324">
         <v>323</v>
       </c>
@@ -27669,11 +27279,8 @@
         <f>'CPP Raw Data'!K292*-1</f>
         <v>0.297414320482845</v>
       </c>
-      <c r="L324">
-        <v>0.248270093</v>
-      </c>
-    </row>
-    <row r="325" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="325" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A325">
         <v>324</v>
       </c>
@@ -27714,11 +27321,8 @@
         <f>'CPP Raw Data'!K293*-1</f>
         <v>0.24119421362789201</v>
       </c>
-      <c r="L325">
-        <v>8.8555665000000006E-2</v>
-      </c>
-    </row>
-    <row r="326" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="326" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A326">
         <v>325</v>
       </c>
@@ -27759,11 +27363,8 @@
         <f>'CPP Raw Data'!K294*-1</f>
         <v>0.21972031841741099</v>
       </c>
-      <c r="L326">
-        <v>0.20681355200000001</v>
-      </c>
-    </row>
-    <row r="327" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="327" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A327">
         <v>326</v>
       </c>
@@ -27804,11 +27405,8 @@
         <f>'CPP Raw Data'!K295*-1</f>
         <v>0.20679035118021699</v>
       </c>
-      <c r="L327">
-        <v>0.16279717899999999</v>
-      </c>
-    </row>
-    <row r="328" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="328" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A328">
         <v>327</v>
       </c>
@@ -27849,11 +27447,8 @@
         <f>'CPP Raw Data'!K296*-1</f>
         <v>0.27476653111180299</v>
       </c>
-      <c r="L328">
-        <v>0.30980207900000001</v>
-      </c>
-    </row>
-    <row r="329" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="329" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A329">
         <v>328</v>
       </c>
@@ -27894,11 +27489,8 @@
         <f>'CPP Raw Data'!K297*-1</f>
         <v>0.26727453289372799</v>
       </c>
-      <c r="L329">
-        <v>0.235658434</v>
-      </c>
-    </row>
-    <row r="330" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="330" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A330">
         <v>329</v>
       </c>
@@ -27939,11 +27531,8 @@
         <f>'CPP Raw Data'!K298*-1</f>
         <v>0.35053047121916298</v>
       </c>
-      <c r="L330">
-        <v>0.30794222399999999</v>
-      </c>
-    </row>
-    <row r="331" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="331" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A331">
         <v>330</v>
       </c>
@@ -27984,11 +27573,8 @@
         <f>'CPP Raw Data'!K299*-1</f>
         <v>0.208968512422092</v>
       </c>
-      <c r="L331">
-        <v>0.18954200900000001</v>
-      </c>
-    </row>
-    <row r="332" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="332" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A332">
         <v>331</v>
       </c>
@@ -28029,11 +27615,8 @@
         <f>'CPP Raw Data'!K300*-1</f>
         <v>0.41690941468981901</v>
       </c>
-      <c r="L332">
-        <v>0.38725499699999999</v>
-      </c>
-    </row>
-    <row r="333" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="333" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A333">
         <v>332</v>
       </c>
@@ -28074,11 +27657,8 @@
         <f>'CPP Raw Data'!K301*-1</f>
         <v>0.43842051702065599</v>
       </c>
-      <c r="L333">
-        <v>0.36173032199999999</v>
-      </c>
-    </row>
-    <row r="334" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="334" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A334">
         <v>333</v>
       </c>
@@ -28119,11 +27699,8 @@
         <f>'CPP Raw Data'!K302*-1</f>
         <v>8.1655107223248494E-2</v>
       </c>
-      <c r="L334">
-        <v>7.2162320000000004E-3</v>
-      </c>
-    </row>
-    <row r="335" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="335" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A335">
         <v>334</v>
       </c>
@@ -28164,11 +27741,8 @@
         <f>'CPP Raw Data'!K303*-1</f>
         <v>0.25815215838385303</v>
       </c>
-      <c r="L335">
-        <v>0.22320478499999999</v>
-      </c>
-    </row>
-    <row r="336" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="336" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A336">
         <v>335</v>
       </c>
@@ -28209,11 +27783,8 @@
         <f>'CPP Raw Data'!K304*-1</f>
         <v>0.34514276207470101</v>
       </c>
-      <c r="L336">
-        <v>0.289972697</v>
-      </c>
-    </row>
-    <row r="337" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="337" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A337">
         <v>336</v>
       </c>
@@ -28254,11 +27825,8 @@
         <f>'CPP Raw Data'!K305*-1</f>
         <v>0.26701423711976702</v>
       </c>
-      <c r="L337">
-        <v>0.25525362699999998</v>
-      </c>
-    </row>
-    <row r="338" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="338" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A338">
         <v>337</v>
       </c>
@@ -28299,11 +27867,8 @@
         <f>'CPP Raw Data'!K306*-1</f>
         <v>0.23921261629282101</v>
       </c>
-      <c r="L338">
-        <v>0.17747057699999999</v>
-      </c>
-    </row>
-    <row r="339" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="339" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A339">
         <v>338</v>
       </c>
@@ -28344,11 +27909,8 @@
         <f>'CPP Raw Data'!K307*-1</f>
         <v>0.375166465871768</v>
       </c>
-      <c r="L339">
-        <v>0.314495152</v>
-      </c>
-    </row>
-    <row r="340" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="340" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A340">
         <v>339</v>
       </c>
@@ -28389,11 +27951,8 @@
         <f>'CPP Raw Data'!K308*-1</f>
         <v>0.25879741669239897</v>
       </c>
-      <c r="L340">
-        <v>0.20139427700000001</v>
-      </c>
-    </row>
-    <row r="341" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="341" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A341">
         <v>340</v>
       </c>
@@ -28434,11 +27993,8 @@
         <f>'CPP Raw Data'!K309*-1</f>
         <v>0.13708215993884801</v>
       </c>
-      <c r="L341">
-        <v>0.14627030299999999</v>
-      </c>
-    </row>
-    <row r="342" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="342" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A342">
         <v>341</v>
       </c>
@@ -28479,11 +28035,8 @@
         <f>'CPP Raw Data'!K310*-1</f>
         <v>0.305405784270395</v>
       </c>
-      <c r="L342">
-        <v>0.236147835</v>
-      </c>
-    </row>
-    <row r="343" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="343" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A343">
         <v>342</v>
       </c>
@@ -28524,11 +28077,8 @@
         <f>'CPP Raw Data'!K311*-1</f>
         <v>0.21284989750739</v>
       </c>
-      <c r="L343">
-        <v>0.18314905200000001</v>
-      </c>
-    </row>
-    <row r="344" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="344" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A344">
         <v>343</v>
       </c>
@@ -28569,11 +28119,8 @@
         <f>'CPP Raw Data'!K312*-1</f>
         <v>0.11939589665653499</v>
       </c>
-      <c r="L344">
-        <v>0.102861145</v>
-      </c>
-    </row>
-    <row r="345" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="345" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A345">
         <v>344</v>
       </c>
@@ -28614,11 +28161,8 @@
         <f>'CPP Raw Data'!K313*-1</f>
         <v>0.26008351011649999</v>
       </c>
-      <c r="L345">
-        <v>0.26479679499999997</v>
-      </c>
-    </row>
-    <row r="346" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="346" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A346">
         <v>345</v>
       </c>
@@ -28659,11 +28203,8 @@
         <f>'CPP Raw Data'!K314*-1</f>
         <v>0.338111459158496</v>
       </c>
-      <c r="L346">
-        <v>0.29571933099999997</v>
-      </c>
-    </row>
-    <row r="347" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="347" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A347">
         <v>346</v>
       </c>
@@ -28704,11 +28245,8 @@
         <f>'CPP Raw Data'!K315*-1</f>
         <v>0.228650606205866</v>
       </c>
-      <c r="L347">
-        <v>0.236845841</v>
-      </c>
-    </row>
-    <row r="348" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="348" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A348">
         <v>347</v>
       </c>
@@ -28749,11 +28287,8 @@
         <f>'CPP Raw Data'!K316*-1</f>
         <v>0.10728579149631801</v>
       </c>
-      <c r="L348">
-        <v>5.6487846000000001E-2</v>
-      </c>
-    </row>
-    <row r="349" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="349" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A349">
         <v>348</v>
       </c>
@@ -28794,11 +28329,8 @@
         <f>'CPP Raw Data'!K317*-1</f>
         <v>0.318603956161221</v>
       </c>
-      <c r="L349">
-        <v>0.31174420200000003</v>
-      </c>
-    </row>
-    <row r="350" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="350" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A350">
         <v>349</v>
       </c>
@@ -28839,11 +28371,8 @@
         <f>'CPP Raw Data'!K318*-1</f>
         <v>0.26081335932244099</v>
       </c>
-      <c r="L350">
-        <v>0.20483553700000001</v>
-      </c>
-    </row>
-    <row r="351" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="351" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A351">
         <v>350</v>
       </c>
@@ -28884,11 +28413,8 @@
         <f>'CPP Raw Data'!K319*-1</f>
         <v>0.34331596485523702</v>
       </c>
-      <c r="L351">
-        <v>0.32442217699999998</v>
-      </c>
-    </row>
-    <row r="352" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="352" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A352">
         <v>351</v>
       </c>
@@ -28929,11 +28455,8 @@
         <f>'CPP Raw Data'!K320*-1</f>
         <v>0.218872449250479</v>
       </c>
-      <c r="L352">
-        <v>0.16244260099999999</v>
-      </c>
-    </row>
-    <row r="353" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="353" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A353">
         <v>352</v>
       </c>
@@ -28974,11 +28497,8 @@
         <f>'CPP Raw Data'!K321*-1</f>
         <v>0.26149581024901303</v>
       </c>
-      <c r="L353">
-        <v>0.23012670900000001</v>
-      </c>
-    </row>
-    <row r="354" spans="1:12" x14ac:dyDescent="0.25">
+    </row>
+    <row r="354" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A354">
         <v>353</v>
       </c>
@@ -29020,7 +28540,7 @@
         <v>0.328055051661226</v>
       </c>
     </row>
-    <row r="355" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A355">
         <v>354</v>
       </c>
@@ -29062,7 +28582,7 @@
         <v>0.29831593877406298</v>
       </c>
     </row>
-    <row r="356" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A356">
         <v>355</v>
       </c>
@@ -29104,7 +28624,7 @@
         <v>0.28033801446235301</v>
       </c>
     </row>
-    <row r="357" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A357">
         <v>356</v>
       </c>
@@ -29146,7 +28666,7 @@
         <v>0.25539344883725901</v>
       </c>
     </row>
-    <row r="358" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A358">
         <v>357</v>
       </c>
@@ -29188,7 +28708,7 @@
         <v>0.24784448672623799</v>
       </c>
     </row>
-    <row r="359" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A359">
         <v>358</v>
       </c>
@@ -29230,7 +28750,7 @@
         <v>0.217184603312816</v>
       </c>
     </row>
-    <row r="360" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A360">
         <v>359</v>
       </c>
@@ -29272,7 +28792,7 @@
         <v>0.27133570797142798</v>
       </c>
     </row>
-    <row r="361" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A361">
         <v>360</v>
       </c>
@@ -29314,7 +28834,7 @@
         <v>0.267052826819345</v>
       </c>
     </row>
-    <row r="362" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A362">
         <v>361</v>
       </c>
@@ -29356,7 +28876,7 @@
         <v>0.36305355577852799</v>
       </c>
     </row>
-    <row r="363" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A363">
         <v>362</v>
       </c>
@@ -29398,7 +28918,7 @@
         <v>0.21396162640070801</v>
       </c>
     </row>
-    <row r="364" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A364">
         <v>363</v>
       </c>
@@ -29440,7 +28960,7 @@
         <v>0.40483171473044299</v>
       </c>
     </row>
-    <row r="365" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A365">
         <v>364</v>
       </c>
@@ -29482,7 +29002,7 @@
         <v>0.43899480502711102</v>
       </c>
     </row>
-    <row r="366" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A366">
         <v>365</v>
       </c>
@@ -29524,7 +29044,7 @@
         <v>7.5390205985237393E-2</v>
       </c>
     </row>
-    <row r="367" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A367">
         <v>366</v>
       </c>
@@ -29566,7 +29086,7 @@
         <v>0.268038081246122</v>
       </c>
     </row>
-    <row r="368" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A368">
         <v>367</v>
       </c>
@@ -31947,6 +31467,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010081FAC630D54E9140B4AB806285961C20" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="4b1ff426f6ab44433fa90133b41c6530">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="0ffb6a14-689f-42ef-a067-675c51ff5d7a" xmlns:ns4="a011b53f-306d-4901-9018-6d427f6237fb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="945afaefde5cbe62288d729dbeb08812" ns3:_="" ns4:_="">
     <xsd:import namespace="0ffb6a14-689f-42ef-a067-675c51ff5d7a"/>
@@ -32163,12 +31689,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D13426F8-84C3-46C1-A03F-03F10DAB276F}">
   <ds:schemaRefs>
@@ -32178,6 +31698,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{082F13FD-C70D-418E-A1E2-3A104DB84F0D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E040864-2A97-4C78-85E7-DAE01F518143}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -32194,13 +31723,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{082F13FD-C70D-418E-A1E2-3A104DB84F0D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>